<commit_message>
Select locally available TYG-50 caster and verify load margin
</commit_message>
<xml_diff>
--- a/cad/amr07/BOM.xlsx
+++ b/cad/amr07/BOM.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="800">
   <si>
     <t xml:space="preserve">AMR-01 / A6　調達BOM</t>
   </si>
@@ -65,7 +65,7 @@
     <t xml:space="preserve">円の途中小計</t>
   </si>
   <si>
-    <t xml:space="preserve">キャスターをナフコ店舗受取498円＋送料0円とする条件。受取店・在庫未確定。販売記録・仮枠・材料消費を含む。</t>
+    <t xml:space="preserve">キャスターをAmazon273円＋既存Prime会員条件の送料0円とする条件。会員ログイン後の最終注文額は未確認。販売記録・仮枠・材料消費を含む。</t>
   </si>
   <si>
     <t xml:space="preserve">USDの途中小計</t>
@@ -116,7 +116,7 @@
     <t xml:space="preserve">タイヤ・キャスター・座金・タイヤ送料を再確認</t>
   </si>
   <si>
-    <t xml:space="preserve">Amazonは再取得できず既存価格。その他は2026-09-21等の既存記録・仮枠。</t>
+    <t xml:space="preserve">フレームのAmazon価格は再取得できず既存価格。キャスターはAmazon販売発送273円を確認。その他は既存記録・仮枠。</t>
   </si>
   <si>
     <t xml:space="preserve">使用数と購入数</t>
@@ -310,7 +310,7 @@
   </si>
   <si>
     <t xml:space="preserve">自在キャスター
-ハンマー420G-R50、径50・取付高65mm</t>
+TRUSCO TYG-50、径50・取付高65mm、穴ピッチ46×35</t>
   </si>
   <si>
     <t xml:space="preserve">1個</t>
@@ -320,11 +320,11 @@
   </si>
   <si>
     <t xml:space="preserve">販売表示・条件付き
-型式維持・個人購入の店舗受取を第一候補</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ナフコ（店舗受取）
-完成品1個。税込498円＋店舗受取送料0円。受取店/在庫未確定、交通費別。ナフコ包装JANは2100256559029、受入時に420G-R50/高さ65/穴ピッチ46×35を照合。</t>
+Amazon販売発送を確認・Prime会員条件の第一候補</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon.co.jp（販売・発送）
+完成品1個、税込273円。Amazon.co.jp販売・発送の出品。既存Prime会員の対象配送を条件に送料0円（公式配送規定）。会員としての最終注文画面は未確認。JAN4989999424980、公称高さ65mm・穴46×35を受入照合。</t>
   </si>
   <si>
     <t xml:space="preserve">P01</t>
@@ -687,11 +687,11 @@
   </si>
   <si>
     <t xml:space="preserve">販売表示・条件付き
-店舗受取の場合のみ0円</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ナフコ（店舗受取）
-商品ページの店舗受取送料無料条件。自宅配送費ではない。受取店・準備日は注文前に確認。</t>
+既存Prime会員の対象配送条件で0円</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon.co.jp（Prime会員条件）
+Amazon公式の会員配送規定を適用する条件。会員ログイン後の最終注文額ではない。非会員の単品購入は別送料。新規会費は含めない。コーナン店舗受取なら商品283円＋受取送料0円。</t>
   </si>
   <si>
     <t xml:space="preserve">S03</t>
@@ -1990,7 +1990,7 @@
     <t xml:space="preserve">CasterTop</t>
   </si>
   <si>
-    <t xml:space="preserve">Hammer420G-R50 | unchanged</t>
+    <t xml:space="preserve">TRUSCO TYG-50 | CasterTop | nominal proxy</t>
   </si>
   <si>
     <t xml:space="preserve">CasterBolt_0</t>
@@ -2044,13 +2044,25 @@
     <t xml:space="preserve">SwivelRace</t>
   </si>
   <si>
+    <t xml:space="preserve">TRUSCO TYG-50 | SwivelRace | nominal proxy</t>
+  </si>
+  <si>
     <t xml:space="preserve">CasterFork</t>
   </si>
   <si>
+    <t xml:space="preserve">TRUSCO TYG-50 | CasterFork | nominal proxy</t>
+  </si>
+  <si>
     <t xml:space="preserve">CasterTire</t>
   </si>
   <si>
+    <t xml:space="preserve">TRUSCO TYG-50 | CasterTire | nominal proxy</t>
+  </si>
+  <si>
     <t xml:space="preserve">CasterCore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRUSCO TYG-50 | CasterCore | nominal proxy</t>
   </si>
   <si>
     <t xml:space="preserve">BatteryCradlePLA</t>
@@ -3266,7 +3278,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">SUMIF(購入品!H5:H44,"JPY",購入品!G5:G44)</f>
-        <v>54414</v>
+        <v>54189</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
@@ -3311,7 +3323,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="10" t="n">
-        <v>8.73314316476638</v>
+        <v>8.74814316476638</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>16</v>
@@ -3698,11 +3710,11 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>498</v>
+        <v>273</v>
       </c>
       <c r="G10" s="19" t="n">
         <f aca="false">E10*F10</f>
-        <v>498</v>
+        <v>273</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>56</v>
@@ -8118,7 +8130,7 @@
         <v>82</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>569</v>
@@ -8127,13 +8139,13 @@
     </row>
     <row r="124" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="6" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B124" s="6" t="s">
         <v>82</v>
       </c>
       <c r="C124" s="6" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D124" s="6" t="s">
         <v>569</v>
@@ -8142,13 +8154,13 @@
     </row>
     <row r="125" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="B125" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>569</v>
@@ -8157,13 +8169,13 @@
     </row>
     <row r="126" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="6" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="B126" s="6" t="s">
         <v>82</v>
       </c>
       <c r="C126" s="6" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="D126" s="6" t="s">
         <v>569</v>
@@ -8172,13 +8184,13 @@
     </row>
     <row r="127" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="B127" s="4" t="s">
         <v>137</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>30</v>
@@ -8187,13 +8199,13 @@
     </row>
     <row r="128" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="6" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="B128" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C128" s="6" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="D128" s="6" t="s">
         <v>418</v>
@@ -8204,13 +8216,13 @@
     </row>
     <row r="129" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="B129" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>418</v>
@@ -8221,13 +8233,13 @@
     </row>
     <row r="130" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="6" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="B130" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="D130" s="6" t="s">
         <v>418</v>
@@ -8238,13 +8250,13 @@
     </row>
     <row r="131" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B131" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>418</v>
@@ -8255,13 +8267,13 @@
     </row>
     <row r="132" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="6" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B132" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="D132" s="6" t="s">
         <v>418</v>
@@ -8272,13 +8284,13 @@
     </row>
     <row r="133" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="B133" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="D133" s="4" t="s">
         <v>418</v>
@@ -8289,13 +8301,13 @@
     </row>
     <row r="134" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="6" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="B134" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C134" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="D134" s="6" t="s">
         <v>418</v>
@@ -8306,13 +8318,13 @@
     </row>
     <row r="135" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B135" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="D135" s="4" t="s">
         <v>418</v>
@@ -8323,13 +8335,13 @@
     </row>
     <row r="136" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="6" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="B136" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C136" s="6" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="D136" s="6" t="s">
         <v>418</v>
@@ -8340,13 +8352,13 @@
     </row>
     <row r="137" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B137" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>418</v>
@@ -8357,13 +8369,13 @@
     </row>
     <row r="138" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="6" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="B138" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C138" s="6" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="D138" s="6" t="s">
         <v>418</v>
@@ -8374,13 +8386,13 @@
     </row>
     <row r="139" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="B139" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D139" s="4" t="s">
         <v>418</v>
@@ -8391,13 +8403,13 @@
     </row>
     <row r="140" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="6" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="B140" s="6" t="s">
         <v>137</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="D140" s="6" t="s">
         <v>30</v>
@@ -8406,13 +8418,13 @@
     </row>
     <row r="141" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="B141" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>418</v>
@@ -8423,13 +8435,13 @@
     </row>
     <row r="142" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="6" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="B142" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C142" s="6" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="D142" s="6" t="s">
         <v>418</v>
@@ -8440,13 +8452,13 @@
     </row>
     <row r="143" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="B143" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="D143" s="4" t="s">
         <v>418</v>
@@ -8457,13 +8469,13 @@
     </row>
     <row r="144" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="6" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="B144" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="D144" s="6" t="s">
         <v>418</v>
@@ -8474,13 +8486,13 @@
     </row>
     <row r="145" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="B145" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D145" s="4" t="s">
         <v>418</v>
@@ -8491,13 +8503,13 @@
     </row>
     <row r="146" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="6" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="B146" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C146" s="6" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D146" s="6" t="s">
         <v>418</v>
@@ -8508,13 +8520,13 @@
     </row>
     <row r="147" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B147" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>418</v>
@@ -8525,13 +8537,13 @@
     </row>
     <row r="148" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="6" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="B148" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C148" s="6" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="D148" s="6" t="s">
         <v>418</v>
@@ -8542,13 +8554,13 @@
     </row>
     <row r="149" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B149" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="D149" s="4" t="s">
         <v>418</v>
@@ -8559,13 +8571,13 @@
     </row>
     <row r="150" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="6" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B150" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C150" s="6" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="D150" s="6" t="s">
         <v>418</v>
@@ -8576,13 +8588,13 @@
     </row>
     <row r="151" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="B151" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="D151" s="4" t="s">
         <v>418</v>
@@ -8593,13 +8605,13 @@
     </row>
     <row r="152" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="6" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="B152" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C152" s="6" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="D152" s="6" t="s">
         <v>418</v>
@@ -8610,13 +8622,13 @@
     </row>
     <row r="153" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B153" s="4" t="s">
         <v>137</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>30</v>
@@ -8625,13 +8637,13 @@
     </row>
     <row r="154" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="6" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="B154" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C154" s="6" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="D154" s="6" t="s">
         <v>418</v>
@@ -8642,13 +8654,13 @@
     </row>
     <row r="155" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="B155" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="D155" s="4" t="s">
         <v>418</v>
@@ -8659,13 +8671,13 @@
     </row>
     <row r="156" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="6" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="B156" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C156" s="6" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="D156" s="6" t="s">
         <v>418</v>
@@ -8676,13 +8688,13 @@
     </row>
     <row r="157" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="B157" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>418</v>
@@ -8693,13 +8705,13 @@
     </row>
     <row r="158" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="6" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="B158" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C158" s="6" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="D158" s="6" t="s">
         <v>418</v>
@@ -8710,13 +8722,13 @@
     </row>
     <row r="159" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="B159" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>418</v>
@@ -8727,13 +8739,13 @@
     </row>
     <row r="160" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="6" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="B160" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C160" s="6" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="D160" s="6" t="s">
         <v>418</v>
@@ -8744,13 +8756,13 @@
     </row>
     <row r="161" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="B161" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="D161" s="4" t="s">
         <v>418</v>
@@ -8761,13 +8773,13 @@
     </row>
     <row r="162" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="6" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="B162" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C162" s="6" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="D162" s="6" t="s">
         <v>418</v>
@@ -8778,13 +8790,13 @@
     </row>
     <row r="163" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="B163" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="D163" s="4" t="s">
         <v>418</v>
@@ -8795,13 +8807,13 @@
     </row>
     <row r="164" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="6" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="B164" s="6" t="s">
         <v>148</v>
       </c>
       <c r="C164" s="6" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="D164" s="6" t="s">
         <v>418</v>
@@ -8812,13 +8824,13 @@
     </row>
     <row r="165" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="B165" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="D165" s="4" t="s">
         <v>418</v>
@@ -8829,13 +8841,13 @@
     </row>
     <row r="166" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="6" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="B166" s="6" t="s">
         <v>151</v>
       </c>
       <c r="C166" s="6" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="D166" s="6" t="s">
         <v>418</v>
@@ -8846,13 +8858,13 @@
     </row>
     <row r="167" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="B167" s="4" t="s">
         <v>151</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="D167" s="4" t="s">
         <v>418</v>
@@ -8863,13 +8875,13 @@
     </row>
     <row r="168" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="6" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="B168" s="6" t="s">
         <v>151</v>
       </c>
       <c r="C168" s="6" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D168" s="6" t="s">
         <v>418</v>
@@ -8880,13 +8892,13 @@
     </row>
     <row r="169" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="B169" s="4" t="s">
         <v>151</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="D169" s="4" t="s">
         <v>418</v>
@@ -8897,13 +8909,13 @@
     </row>
     <row r="170" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="6" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="B170" s="6" t="s">
         <v>151</v>
       </c>
       <c r="C170" s="6" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="D170" s="6" t="s">
         <v>418</v>
@@ -8914,13 +8926,13 @@
     </row>
     <row r="171" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B171" s="4" t="s">
         <v>151</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="D171" s="4" t="s">
         <v>418</v>
@@ -8931,13 +8943,13 @@
     </row>
     <row r="172" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="6" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="B172" s="6" t="s">
         <v>111</v>
       </c>
       <c r="C172" s="6" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="D172" s="6" t="s">
         <v>403</v>
@@ -8946,13 +8958,13 @@
     </row>
     <row r="173" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="B173" s="4" t="s">
         <v>116</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="D173" s="4" t="s">
         <v>403</v>
@@ -8961,13 +8973,13 @@
     </row>
     <row r="174" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="6" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="B174" s="6" t="s">
         <v>116</v>
       </c>
       <c r="C174" s="6" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="D174" s="6" t="s">
         <v>403</v>
@@ -8976,13 +8988,13 @@
     </row>
     <row r="175" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B175" s="4" t="s">
         <v>116</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="D175" s="4" t="s">
         <v>403</v>
@@ -8991,13 +9003,13 @@
     </row>
     <row r="176" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="6" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="B176" s="6" t="s">
         <v>116</v>
       </c>
       <c r="C176" s="6" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="D176" s="6" t="s">
         <v>403</v>
@@ -9006,13 +9018,13 @@
     </row>
     <row r="177" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="B177" s="4" t="s">
         <v>116</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="D177" s="4" t="s">
         <v>403</v>
@@ -9021,13 +9033,13 @@
     </row>
     <row r="178" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="6" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="B178" s="6" t="s">
         <v>116</v>
       </c>
       <c r="C178" s="6" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="D178" s="6" t="s">
         <v>403</v>
@@ -9036,13 +9048,13 @@
     </row>
     <row r="179" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="B179" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="D179" s="4" t="s">
         <v>418</v>
@@ -9053,13 +9065,13 @@
     </row>
     <row r="180" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="6" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B180" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C180" s="6" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="D180" s="6" t="s">
         <v>418</v>
@@ -9070,13 +9082,13 @@
     </row>
     <row r="181" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="B181" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="D181" s="4" t="s">
         <v>418</v>
@@ -9087,13 +9099,13 @@
     </row>
     <row r="182" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="6" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B182" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C182" s="6" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="D182" s="6" t="s">
         <v>418</v>
@@ -9104,13 +9116,13 @@
     </row>
     <row r="183" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="4" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="B183" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="D183" s="4" t="s">
         <v>418</v>
@@ -9121,13 +9133,13 @@
     </row>
     <row r="184" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="6" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="B184" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C184" s="6" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="D184" s="6" t="s">
         <v>418</v>
@@ -9138,13 +9150,13 @@
     </row>
     <row r="185" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="4" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="B185" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="D185" s="4" t="s">
         <v>418</v>
@@ -9155,13 +9167,13 @@
     </row>
     <row r="186" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="6" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="B186" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C186" s="6" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D186" s="6" t="s">
         <v>418</v>
@@ -9172,13 +9184,13 @@
     </row>
     <row r="187" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="4" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="B187" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="D187" s="4" t="s">
         <v>418</v>
@@ -9189,13 +9201,13 @@
     </row>
     <row r="188" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="6" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B188" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C188" s="6" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="D188" s="6" t="s">
         <v>418</v>
@@ -9206,13 +9218,13 @@
     </row>
     <row r="189" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="4" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="B189" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="D189" s="4" t="s">
         <v>418</v>
@@ -9223,13 +9235,13 @@
     </row>
     <row r="190" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="6" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="B190" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C190" s="6" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="D190" s="6" t="s">
         <v>418</v>
@@ -9240,13 +9252,13 @@
     </row>
     <row r="191" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="4" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="B191" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="D191" s="4" t="s">
         <v>418</v>
@@ -9257,13 +9269,13 @@
     </row>
     <row r="192" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="6" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="B192" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C192" s="6" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="D192" s="6" t="s">
         <v>418</v>
@@ -9274,13 +9286,13 @@
     </row>
     <row r="193" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="4" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="B193" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="D193" s="4" t="s">
         <v>418</v>
@@ -9291,13 +9303,13 @@
     </row>
     <row r="194" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="6" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B194" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C194" s="6" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="D194" s="6" t="s">
         <v>418</v>
@@ -9308,13 +9320,13 @@
     </row>
     <row r="195" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="4" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="B195" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="D195" s="4" t="s">
         <v>418</v>
@@ -9325,13 +9337,13 @@
     </row>
     <row r="196" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="6" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="B196" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C196" s="6" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="D196" s="6" t="s">
         <v>418</v>
@@ -9342,13 +9354,13 @@
     </row>
     <row r="197" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="4" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="B197" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="D197" s="4" t="s">
         <v>418</v>
@@ -9359,13 +9371,13 @@
     </row>
     <row r="198" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="6" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="B198" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C198" s="6" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="D198" s="6" t="s">
         <v>418</v>
@@ -9376,13 +9388,13 @@
     </row>
     <row r="199" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="4" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="B199" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="D199" s="4" t="s">
         <v>418</v>
@@ -9393,13 +9405,13 @@
     </row>
     <row r="200" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="6" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="B200" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C200" s="6" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="D200" s="6" t="s">
         <v>418</v>
@@ -9410,13 +9422,13 @@
     </row>
     <row r="201" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="4" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="B201" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="D201" s="4" t="s">
         <v>418</v>
@@ -9427,13 +9439,13 @@
     </row>
     <row r="202" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="6" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="B202" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C202" s="6" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="D202" s="6" t="s">
         <v>418</v>
@@ -9444,13 +9456,13 @@
     </row>
     <row r="203" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="4" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="B203" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D203" s="4" t="s">
         <v>418</v>
@@ -9461,13 +9473,13 @@
     </row>
     <row r="204" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="6" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="B204" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C204" s="6" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="D204" s="6" t="s">
         <v>418</v>
@@ -9478,13 +9490,13 @@
     </row>
     <row r="205" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="4" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B205" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="D205" s="4" t="s">
         <v>418</v>
@@ -9495,13 +9507,13 @@
     </row>
     <row r="206" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="6" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="B206" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C206" s="6" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="D206" s="6" t="s">
         <v>418</v>
@@ -9512,13 +9524,13 @@
     </row>
     <row r="207" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="4" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="B207" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="D207" s="4" t="s">
         <v>418</v>
@@ -9529,13 +9541,13 @@
     </row>
     <row r="208" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="6" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="B208" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C208" s="6" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="D208" s="6" t="s">
         <v>418</v>
@@ -9546,13 +9558,13 @@
     </row>
     <row r="209" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="4" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="B209" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="D209" s="4" t="s">
         <v>418</v>
@@ -9563,13 +9575,13 @@
     </row>
     <row r="210" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="6" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="B210" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C210" s="6" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="D210" s="6" t="s">
         <v>418</v>
@@ -9580,13 +9592,13 @@
     </row>
     <row r="211" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="4" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="B211" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="D211" s="4" t="s">
         <v>418</v>
@@ -9597,13 +9609,13 @@
     </row>
     <row r="212" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="6" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="B212" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C212" s="6" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="D212" s="6" t="s">
         <v>418</v>
@@ -9614,13 +9626,13 @@
     </row>
     <row r="213" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="4" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="B213" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C213" s="4" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="D213" s="4" t="s">
         <v>418</v>
@@ -9631,13 +9643,13 @@
     </row>
     <row r="214" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="6" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="B214" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C214" s="6" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="D214" s="6" t="s">
         <v>418</v>
@@ -9648,13 +9660,13 @@
     </row>
     <row r="215" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="4" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="B215" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C215" s="4" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="D215" s="4" t="s">
         <v>418</v>
@@ -9665,13 +9677,13 @@
     </row>
     <row r="216" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="6" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="B216" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C216" s="6" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="D216" s="6" t="s">
         <v>418</v>
@@ -9682,13 +9694,13 @@
     </row>
     <row r="217" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="4" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="B217" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="D217" s="4" t="s">
         <v>418</v>
@@ -9699,13 +9711,13 @@
     </row>
     <row r="218" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="6" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="B218" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C218" s="6" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="D218" s="6" t="s">
         <v>418</v>
@@ -9716,13 +9728,13 @@
     </row>
     <row r="219" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="4" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="B219" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="D219" s="4" t="s">
         <v>418</v>
@@ -9733,13 +9745,13 @@
     </row>
     <row r="220" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="6" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="B220" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C220" s="6" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="D220" s="6" t="s">
         <v>418</v>
@@ -9750,13 +9762,13 @@
     </row>
     <row r="221" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="4" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="B221" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="D221" s="4" t="s">
         <v>418</v>
@@ -9767,13 +9779,13 @@
     </row>
     <row r="222" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="6" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="B222" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C222" s="6" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="D222" s="6" t="s">
         <v>418</v>
@@ -9784,13 +9796,13 @@
     </row>
     <row r="223" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="4" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="B223" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="D223" s="4" t="s">
         <v>418</v>
@@ -9801,13 +9813,13 @@
     </row>
     <row r="224" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="6" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="B224" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C224" s="6" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="D224" s="6" t="s">
         <v>418</v>
@@ -9818,13 +9830,13 @@
     </row>
     <row r="225" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="4" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="B225" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="D225" s="4" t="s">
         <v>418</v>
@@ -9835,13 +9847,13 @@
     </row>
     <row r="226" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="6" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="B226" s="6" t="s">
         <v>126</v>
       </c>
       <c r="C226" s="6" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="D226" s="6" t="s">
         <v>418</v>

</xml_diff>